<commit_message>
Realizacion de notificaciones para ventanas, y correcciones
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO SUM COTIZACIONES.xlsx
+++ b/storage/app/templates/FORMATO SUM COTIZACIONES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA-OFICIAL-AGARCORP\storage\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CB62F8-5943-4F56-AAB7-902DC74B3181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEEE20FB-77F5-4AC5-A3FE-E638F8D686B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{309D63E5-5CD5-46E5-9FEC-D63E43A25BAB}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8964" xr2:uid="{309D63E5-5CD5-46E5-9FEC-D63E43A25BAB}"/>
   </bookViews>
   <sheets>
     <sheet name="REFERENCIA SUMARIO" sheetId="1" r:id="rId1"/>
@@ -314,42 +314,6 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>FIRMA:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">                                               </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">   FECHA:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> {{elaborado_fecha}}</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">REVISADO POR: </t>
     </r>
     <r>
@@ -381,6 +345,36 @@
     </r>
   </si>
   <si>
+    <t>{{procedencia_importado}}</t>
+  </si>
+  <si>
+    <t>{{procedencia_local}}</t>
+  </si>
+  <si>
+    <t>{{tipo_orden_compra}}</t>
+  </si>
+  <si>
+    <t>{{tipo_orden_servicios}}</t>
+  </si>
+  <si>
+    <t>{{prioridad_mejor_precio}}</t>
+  </si>
+  <si>
+    <t>{{prioridad_mejor_servicio}}</t>
+  </si>
+  <si>
+    <t>{{item}}</t>
+  </si>
+  <si>
+    <t>{{descripcion}}</t>
+  </si>
+  <si>
+    <t>{{unidad_medida}}</t>
+  </si>
+  <si>
+    <t>{{cantidad}}</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -388,7 +382,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">FIRMA:           </t>
+      <t>FIRMA:</t>
     </r>
     <r>
       <rPr>
@@ -396,7 +390,60 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">                                                           </t>
+      <t xml:space="preserve"> {{firma_aprobado}}                                         </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> FECHA:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> {{elaborado_fecha}}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">FIRMA: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">{{firma_revisado}}  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">                                              </t>
     </r>
     <r>
       <rPr>
@@ -415,36 +462,6 @@
       </rPr>
       <t xml:space="preserve"> {{revisado_fecha}}</t>
     </r>
-  </si>
-  <si>
-    <t>{{procedencia_importado}}</t>
-  </si>
-  <si>
-    <t>{{procedencia_local}}</t>
-  </si>
-  <si>
-    <t>{{tipo_orden_compra}}</t>
-  </si>
-  <si>
-    <t>{{tipo_orden_servicios}}</t>
-  </si>
-  <si>
-    <t>{{prioridad_mejor_precio}}</t>
-  </si>
-  <si>
-    <t>{{prioridad_mejor_servicio}}</t>
-  </si>
-  <si>
-    <t>{{item}}</t>
-  </si>
-  <si>
-    <t>{{descripcion}}</t>
-  </si>
-  <si>
-    <t>{{unidad_medida}}</t>
-  </si>
-  <si>
-    <t>{{cantidad}}</t>
   </si>
 </sst>
 </file>
@@ -509,18 +526,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -994,7 +1005,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="134">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
@@ -1022,80 +1033,59 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="16" fontId="2" fillId="3" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="16" fontId="2" fillId="2" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1145,6 +1135,205 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="16"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="8"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="8"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1216,190 +1405,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="16"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="8"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="8"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2819,82 +2824,82 @@
   <sheetData>
     <row r="2" spans="2:16" ht="15.6" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="52"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="58" t="s">
+      <c r="B3" s="110"/>
+      <c r="C3" s="111"/>
+      <c r="D3" s="116" t="s">
         <v>0</v>
       </c>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="60"/>
-      <c r="N3" s="67" t="s">
+      <c r="E3" s="117"/>
+      <c r="F3" s="117"/>
+      <c r="G3" s="117"/>
+      <c r="H3" s="117"/>
+      <c r="I3" s="117"/>
+      <c r="J3" s="117"/>
+      <c r="K3" s="117"/>
+      <c r="L3" s="117"/>
+      <c r="M3" s="118"/>
+      <c r="N3" s="125" t="s">
         <v>1</v>
       </c>
-      <c r="O3" s="68"/>
-      <c r="P3" s="69"/>
+      <c r="O3" s="126"/>
+      <c r="P3" s="127"/>
     </row>
     <row r="4" spans="2:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="54"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="62"/>
-      <c r="L4" s="62"/>
-      <c r="M4" s="63"/>
-      <c r="N4" s="70" t="s">
+      <c r="B4" s="112"/>
+      <c r="C4" s="113"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="120"/>
+      <c r="F4" s="120"/>
+      <c r="G4" s="120"/>
+      <c r="H4" s="120"/>
+      <c r="I4" s="120"/>
+      <c r="J4" s="120"/>
+      <c r="K4" s="120"/>
+      <c r="L4" s="120"/>
+      <c r="M4" s="121"/>
+      <c r="N4" s="128" t="s">
         <v>2</v>
       </c>
-      <c r="O4" s="71"/>
-      <c r="P4" s="72"/>
+      <c r="O4" s="129"/>
+      <c r="P4" s="130"/>
     </row>
     <row r="5" spans="2:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="54"/>
-      <c r="C5" s="55"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="62"/>
-      <c r="F5" s="62"/>
-      <c r="G5" s="62"/>
-      <c r="H5" s="62"/>
-      <c r="I5" s="62"/>
-      <c r="J5" s="62"/>
-      <c r="K5" s="62"/>
-      <c r="L5" s="62"/>
-      <c r="M5" s="63"/>
-      <c r="N5" s="70" t="s">
+      <c r="B5" s="112"/>
+      <c r="C5" s="113"/>
+      <c r="D5" s="119"/>
+      <c r="E5" s="120"/>
+      <c r="F5" s="120"/>
+      <c r="G5" s="120"/>
+      <c r="H5" s="120"/>
+      <c r="I5" s="120"/>
+      <c r="J5" s="120"/>
+      <c r="K5" s="120"/>
+      <c r="L5" s="120"/>
+      <c r="M5" s="121"/>
+      <c r="N5" s="128" t="s">
         <v>3</v>
       </c>
-      <c r="O5" s="71"/>
-      <c r="P5" s="72"/>
+      <c r="O5" s="129"/>
+      <c r="P5" s="130"/>
     </row>
     <row r="6" spans="2:16" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="56"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="64"/>
-      <c r="E6" s="65"/>
-      <c r="F6" s="65"/>
-      <c r="G6" s="65"/>
-      <c r="H6" s="65"/>
-      <c r="I6" s="65"/>
-      <c r="J6" s="65"/>
-      <c r="K6" s="65"/>
-      <c r="L6" s="65"/>
-      <c r="M6" s="66"/>
-      <c r="N6" s="73" t="s">
+      <c r="B6" s="114"/>
+      <c r="C6" s="115"/>
+      <c r="D6" s="122"/>
+      <c r="E6" s="123"/>
+      <c r="F6" s="123"/>
+      <c r="G6" s="123"/>
+      <c r="H6" s="123"/>
+      <c r="I6" s="123"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
+      <c r="L6" s="123"/>
+      <c r="M6" s="124"/>
+      <c r="N6" s="131" t="s">
         <v>4</v>
       </c>
-      <c r="O6" s="74"/>
-      <c r="P6" s="75"/>
+      <c r="O6" s="132"/>
+      <c r="P6" s="133"/>
     </row>
     <row r="7" spans="2:16" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
@@ -2913,36 +2918,36 @@
       <c r="P7" s="5"/>
     </row>
     <row r="8" spans="2:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="95" t="s">
+      <c r="B8" s="83" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="96"/>
-      <c r="D8" s="97" t="s">
+      <c r="C8" s="84"/>
+      <c r="D8" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="97"/>
-      <c r="F8" s="97"/>
-      <c r="G8" s="97"/>
+      <c r="E8" s="85"/>
+      <c r="F8" s="85"/>
+      <c r="G8" s="85"/>
       <c r="H8" s="6"/>
       <c r="I8" s="7"/>
       <c r="M8" s="8" t="s">
         <v>6</v>
       </c>
       <c r="N8" s="8"/>
-      <c r="O8" s="98" t="s">
+      <c r="O8" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="P8" s="99"/>
+      <c r="P8" s="87"/>
     </row>
     <row r="9" spans="2:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2"/>
-      <c r="E9" s="100" t="s">
+      <c r="E9" s="88" t="s">
         <v>28</v>
       </c>
-      <c r="F9" s="100"/>
-      <c r="G9" s="100"/>
-      <c r="H9" s="100"/>
-      <c r="I9" s="100"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
       <c r="P9" s="9"/>
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.25">
@@ -2950,27 +2955,27 @@
         <v>7</v>
       </c>
       <c r="D10" s="10"/>
-      <c r="E10" s="101"/>
-      <c r="F10" s="101"/>
-      <c r="G10" s="101"/>
-      <c r="H10" s="101"/>
-      <c r="I10" s="101"/>
-      <c r="J10" s="102" t="s">
+      <c r="E10" s="89"/>
+      <c r="F10" s="89"/>
+      <c r="G10" s="89"/>
+      <c r="H10" s="89"/>
+      <c r="I10" s="89"/>
+      <c r="J10" s="90" t="s">
         <v>8</v>
       </c>
-      <c r="K10" s="102"/>
-      <c r="L10" s="102"/>
-      <c r="M10" s="102"/>
+      <c r="K10" s="90"/>
+      <c r="L10" s="90"/>
+      <c r="M10" s="90"/>
       <c r="N10" s="8"/>
       <c r="O10" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="P10" s="11"/>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B11" s="2"/>
       <c r="O11" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="P11" s="11"/>
     </row>
@@ -2979,67 +2984,67 @@
       <c r="P12" s="9"/>
     </row>
     <row r="13" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="76" t="s">
+      <c r="B13" s="91" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="77" t="s">
+      <c r="C13" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="78"/>
-      <c r="E13" s="79"/>
-      <c r="F13" s="86" t="s">
+      <c r="D13" s="93"/>
+      <c r="E13" s="94"/>
+      <c r="F13" s="101" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="89" t="s">
+      <c r="G13" s="104" t="s">
         <v>12</v>
       </c>
-      <c r="H13" s="92" t="s">
+      <c r="H13" s="107" t="s">
         <v>13</v>
       </c>
-      <c r="I13" s="93"/>
-      <c r="J13" s="94"/>
-      <c r="K13" s="106" t="s">
+      <c r="I13" s="108"/>
+      <c r="J13" s="109"/>
+      <c r="K13" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="L13" s="107"/>
-      <c r="M13" s="108"/>
-      <c r="N13" s="109" t="s">
+      <c r="L13" s="71"/>
+      <c r="M13" s="72"/>
+      <c r="N13" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="O13" s="110"/>
-      <c r="P13" s="111"/>
+      <c r="O13" s="74"/>
+      <c r="P13" s="75"/>
     </row>
     <row r="14" spans="2:16" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="76"/>
-      <c r="C14" s="80"/>
-      <c r="D14" s="81"/>
-      <c r="E14" s="82"/>
-      <c r="F14" s="87"/>
-      <c r="G14" s="90"/>
-      <c r="H14" s="112" t="s">
+      <c r="B14" s="91"/>
+      <c r="C14" s="95"/>
+      <c r="D14" s="96"/>
+      <c r="E14" s="97"/>
+      <c r="F14" s="102"/>
+      <c r="G14" s="105"/>
+      <c r="H14" s="76" t="s">
         <v>29</v>
       </c>
-      <c r="I14" s="113"/>
-      <c r="J14" s="114"/>
-      <c r="K14" s="112" t="s">
+      <c r="I14" s="77"/>
+      <c r="J14" s="78"/>
+      <c r="K14" s="76" t="s">
         <v>31</v>
       </c>
-      <c r="L14" s="113"/>
-      <c r="M14" s="114"/>
-      <c r="N14" s="112" t="s">
+      <c r="L14" s="77"/>
+      <c r="M14" s="78"/>
+      <c r="N14" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="O14" s="113"/>
-      <c r="P14" s="114"/>
+      <c r="O14" s="77"/>
+      <c r="P14" s="78"/>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B15" s="76"/>
-      <c r="C15" s="80"/>
-      <c r="D15" s="81"/>
-      <c r="E15" s="82"/>
-      <c r="F15" s="87"/>
-      <c r="G15" s="90"/>
-      <c r="H15" s="115" t="s">
+      <c r="B15" s="91"/>
+      <c r="C15" s="95"/>
+      <c r="D15" s="96"/>
+      <c r="E15" s="97"/>
+      <c r="F15" s="102"/>
+      <c r="G15" s="105"/>
+      <c r="H15" s="79" t="s">
         <v>14</v>
       </c>
       <c r="I15" s="12" t="s">
@@ -3048,137 +3053,137 @@
       <c r="J15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="K15" s="117" t="s">
+      <c r="K15" s="81" t="s">
         <v>14</v>
       </c>
-      <c r="L15" s="13" t="s">
+      <c r="L15" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="M15" s="14" t="s">
+      <c r="M15" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="N15" s="117" t="s">
+      <c r="N15" s="81" t="s">
         <v>14</v>
       </c>
-      <c r="O15" s="15" t="s">
+      <c r="O15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="P15" s="16" t="s">
+      <c r="P15" s="48" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B16" s="76"/>
-      <c r="C16" s="83"/>
-      <c r="D16" s="84"/>
-      <c r="E16" s="85"/>
-      <c r="F16" s="88"/>
-      <c r="G16" s="91"/>
-      <c r="H16" s="116"/>
-      <c r="I16" s="17" t="s">
+      <c r="B16" s="91"/>
+      <c r="C16" s="98"/>
+      <c r="D16" s="99"/>
+      <c r="E16" s="100"/>
+      <c r="F16" s="103"/>
+      <c r="G16" s="106"/>
+      <c r="H16" s="80"/>
+      <c r="I16" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="J16" s="17" t="s">
+      <c r="J16" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="K16" s="118"/>
-      <c r="L16" s="18" t="s">
+      <c r="K16" s="82"/>
+      <c r="L16" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="M16" s="19" t="s">
+      <c r="M16" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="N16" s="118"/>
-      <c r="O16" s="18" t="s">
+      <c r="N16" s="82"/>
+      <c r="O16" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="P16" s="20" t="s">
+      <c r="P16" s="50" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="17" spans="2:19" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="21" t="s">
+      <c r="B17" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D17" s="68"/>
+      <c r="E17" s="69"/>
+      <c r="F17" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="103" t="s">
+      <c r="G17" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D17" s="104"/>
-      <c r="E17" s="105"/>
-      <c r="F17" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G17" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="H17" s="27" t="s">
+      <c r="H17" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="I17" s="26" t="s">
+      <c r="I17" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J17" s="26" t="s">
+      <c r="J17" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K17" s="28" t="s">
+      <c r="K17" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L17" s="24" t="s">
+      <c r="L17" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="M17" s="24" t="s">
+      <c r="M17" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="N17" s="28" t="s">
+      <c r="N17" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O17" s="135" t="s">
+      <c r="O17" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="P17" s="25" t="s">
+      <c r="P17" s="18" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="18" spans="2:19" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D18" s="68"/>
+      <c r="E18" s="69"/>
+      <c r="F18" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C18" s="103" t="s">
+      <c r="G18" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D18" s="104"/>
-      <c r="E18" s="105"/>
-      <c r="F18" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G18" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="H18" s="27" t="s">
+      <c r="H18" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="I18" s="26" t="s">
+      <c r="I18" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J18" s="26" t="s">
+      <c r="J18" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K18" s="28" t="s">
+      <c r="K18" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L18" s="24" t="s">
+      <c r="L18" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="M18" s="24" t="s">
+      <c r="M18" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="N18" s="28" t="s">
+      <c r="N18" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O18" s="135" t="s">
+      <c r="O18" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="P18" s="25" t="s">
+      <c r="P18" s="18" t="s">
         <v>41</v>
       </c>
       <c r="S18" s="1" t="s">
@@ -3186,390 +3191,390 @@
       </c>
     </row>
     <row r="19" spans="2:19" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19" s="68"/>
+      <c r="E19" s="69"/>
+      <c r="F19" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C19" s="103" t="s">
+      <c r="G19" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="104"/>
-      <c r="E19" s="105"/>
-      <c r="F19" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G19" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="H19" s="27" t="s">
+      <c r="H19" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="I19" s="26" t="s">
+      <c r="I19" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J19" s="26" t="s">
+      <c r="J19" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K19" s="28" t="s">
+      <c r="K19" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L19" s="24" t="s">
+      <c r="L19" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="M19" s="24" t="s">
+      <c r="M19" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="N19" s="28" t="s">
+      <c r="N19" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O19" s="135" t="s">
+      <c r="O19" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="P19" s="25" t="s">
+      <c r="P19" s="18" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D20" s="68"/>
+      <c r="E20" s="69"/>
+      <c r="F20" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C20" s="103" t="s">
+      <c r="G20" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D20" s="104"/>
-      <c r="E20" s="105"/>
-      <c r="F20" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G20" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="H20" s="27" t="s">
+      <c r="H20" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="I20" s="26" t="s">
+      <c r="I20" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J20" s="26" t="s">
+      <c r="J20" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K20" s="28" t="s">
+      <c r="K20" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L20" s="24" t="s">
+      <c r="L20" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="M20" s="24" t="s">
+      <c r="M20" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="N20" s="28" t="s">
+      <c r="N20" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O20" s="135" t="s">
+      <c r="O20" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="P20" s="25" t="s">
+      <c r="P20" s="18" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="2:19" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="68"/>
+      <c r="E21" s="69"/>
+      <c r="F21" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="103" t="s">
+      <c r="G21" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D21" s="104"/>
-      <c r="E21" s="105"/>
-      <c r="F21" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G21" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="H21" s="27" t="s">
+      <c r="H21" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="I21" s="26" t="s">
+      <c r="I21" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J21" s="26" t="s">
+      <c r="J21" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K21" s="28" t="s">
+      <c r="K21" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L21" s="24" t="s">
+      <c r="L21" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="M21" s="24" t="s">
+      <c r="M21" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="N21" s="28" t="s">
+      <c r="N21" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O21" s="135" t="s">
+      <c r="O21" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="P21" s="25" t="s">
+      <c r="P21" s="18" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="22" spans="2:19" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" s="68"/>
+      <c r="E22" s="69"/>
+      <c r="F22" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="103" t="s">
+      <c r="G22" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D22" s="104"/>
-      <c r="E22" s="105"/>
-      <c r="F22" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G22" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="H22" s="27" t="s">
+      <c r="H22" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="I22" s="26" t="s">
+      <c r="I22" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J22" s="26" t="s">
+      <c r="J22" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K22" s="28" t="s">
+      <c r="K22" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L22" s="24" t="s">
+      <c r="L22" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="M22" s="24" t="s">
+      <c r="M22" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="N22" s="28" t="s">
+      <c r="N22" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O22" s="135" t="s">
+      <c r="O22" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="P22" s="25" t="s">
+      <c r="P22" s="18" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="23" spans="2:19" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D23" s="68"/>
+      <c r="E23" s="69"/>
+      <c r="F23" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="103" t="s">
+      <c r="G23" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D23" s="104"/>
-      <c r="E23" s="105"/>
-      <c r="F23" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G23" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="H23" s="27" t="s">
+      <c r="H23" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="I23" s="26" t="s">
+      <c r="I23" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J23" s="26" t="s">
+      <c r="J23" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K23" s="28" t="s">
+      <c r="K23" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L23" s="24" t="s">
+      <c r="L23" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="M23" s="24" t="s">
+      <c r="M23" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="N23" s="28" t="s">
+      <c r="N23" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O23" s="135" t="s">
+      <c r="O23" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="P23" s="25" t="s">
+      <c r="P23" s="18" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="24" spans="2:19" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D24" s="68"/>
+      <c r="E24" s="69"/>
+      <c r="F24" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="103" t="s">
+      <c r="G24" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D24" s="104"/>
-      <c r="E24" s="105"/>
-      <c r="F24" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G24" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="H24" s="27" t="s">
+      <c r="H24" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="I24" s="26" t="s">
+      <c r="I24" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J24" s="26" t="s">
+      <c r="J24" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K24" s="28" t="s">
+      <c r="K24" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L24" s="24" t="s">
+      <c r="L24" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="M24" s="24" t="s">
+      <c r="M24" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="N24" s="28" t="s">
+      <c r="N24" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O24" s="135" t="s">
+      <c r="O24" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="P24" s="25" t="s">
+      <c r="P24" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="R24" s="29"/>
+      <c r="R24" s="22"/>
     </row>
     <row r="25" spans="2:19" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C25" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D25" s="68"/>
+      <c r="E25" s="69"/>
+      <c r="F25" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="103" t="s">
+      <c r="G25" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="104"/>
-      <c r="E25" s="105"/>
-      <c r="F25" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G25" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="H25" s="27" t="s">
+      <c r="H25" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="I25" s="26" t="s">
+      <c r="I25" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J25" s="26" t="s">
+      <c r="J25" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K25" s="28" t="s">
+      <c r="K25" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L25" s="24" t="s">
+      <c r="L25" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="M25" s="24" t="s">
+      <c r="M25" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="N25" s="28" t="s">
+      <c r="N25" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O25" s="135" t="s">
+      <c r="O25" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="P25" s="25" t="s">
+      <c r="P25" s="18" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="26" spans="2:19" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D26" s="68"/>
+      <c r="E26" s="69"/>
+      <c r="F26" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="103" t="s">
+      <c r="G26" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D26" s="104"/>
-      <c r="E26" s="105"/>
-      <c r="F26" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G26" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="H26" s="27" t="s">
+      <c r="H26" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="I26" s="26" t="s">
+      <c r="I26" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J26" s="26" t="s">
+      <c r="J26" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K26" s="28" t="s">
+      <c r="K26" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L26" s="24" t="s">
+      <c r="L26" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="M26" s="24" t="s">
+      <c r="M26" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="N26" s="28" t="s">
+      <c r="N26" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O26" s="135" t="s">
+      <c r="O26" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="P26" s="25" t="s">
+      <c r="P26" s="18" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="27" spans="2:19" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D27" s="68"/>
+      <c r="E27" s="69"/>
+      <c r="F27" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C27" s="103" t="s">
+      <c r="G27" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D27" s="104"/>
-      <c r="E27" s="105"/>
-      <c r="F27" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G27" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="H27" s="27" t="s">
+      <c r="H27" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="I27" s="26" t="s">
+      <c r="I27" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J27" s="26" t="s">
+      <c r="J27" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K27" s="28" t="s">
+      <c r="K27" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L27" s="24" t="s">
+      <c r="L27" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="M27" s="24" t="s">
+      <c r="M27" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="N27" s="28" t="s">
+      <c r="N27" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O27" s="135" t="s">
+      <c r="O27" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="P27" s="25" t="s">
+      <c r="P27" s="18" t="s">
         <v>41</v>
       </c>
     </row>
@@ -3582,68 +3587,68 @@
       <c r="B29" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G29" s="30"/>
-      <c r="H29" s="30"/>
-      <c r="I29" s="31" t="s">
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="J29" s="32" t="s">
+      <c r="J29" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="K29" s="33"/>
-      <c r="L29" s="34"/>
-      <c r="M29" s="32" t="s">
+      <c r="K29" s="26"/>
+      <c r="L29" s="27"/>
+      <c r="M29" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="N29" s="33"/>
-      <c r="O29" s="34"/>
-      <c r="P29" s="35" t="s">
+      <c r="N29" s="26"/>
+      <c r="O29" s="27"/>
+      <c r="P29" s="28" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="30" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="2"/>
       <c r="C30" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D30" s="10"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="30"/>
-      <c r="I30" s="31" t="s">
+      <c r="G30" s="23"/>
+      <c r="H30" s="23"/>
+      <c r="I30" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="J30" s="36" t="s">
+      <c r="J30" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="K30" s="37"/>
-      <c r="M30" s="36" t="s">
+      <c r="K30" s="30"/>
+      <c r="M30" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="N30" s="37"/>
-      <c r="P30" s="38" t="s">
+      <c r="N30" s="30"/>
+      <c r="P30" s="31" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="31" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="2"/>
       <c r="C31" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D31" s="10"/>
-      <c r="G31" s="30"/>
-      <c r="H31" s="30"/>
-      <c r="I31" s="31" t="s">
+      <c r="G31" s="23"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J31" s="39" t="s">
+      <c r="J31" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="K31" s="40"/>
-      <c r="M31" s="39" t="s">
+      <c r="K31" s="33"/>
+      <c r="M31" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="N31" s="40"/>
-      <c r="P31" s="41" t="s">
+      <c r="N31" s="33"/>
+      <c r="P31" s="34" t="s">
         <v>47</v>
       </c>
     </row>
@@ -3652,149 +3657,149 @@
       <c r="P32" s="9"/>
     </row>
     <row r="33" spans="2:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="128" t="s">
+      <c r="B33" s="66" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="124"/>
-      <c r="D33" s="124"/>
-      <c r="E33" s="124"/>
-      <c r="F33" s="124"/>
-      <c r="G33" s="124"/>
-      <c r="H33" s="124"/>
-      <c r="I33" s="124"/>
-      <c r="J33" s="125"/>
-      <c r="K33" s="42"/>
-      <c r="L33" s="121" t="s">
+      <c r="C33" s="62"/>
+      <c r="D33" s="62"/>
+      <c r="E33" s="62"/>
+      <c r="F33" s="62"/>
+      <c r="G33" s="62"/>
+      <c r="H33" s="62"/>
+      <c r="I33" s="62"/>
+      <c r="J33" s="63"/>
+      <c r="K33" s="35"/>
+      <c r="L33" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="M33" s="121"/>
-      <c r="N33" s="121"/>
-      <c r="O33" s="121"/>
-      <c r="P33" s="122"/>
+      <c r="M33" s="59"/>
+      <c r="N33" s="59"/>
+      <c r="O33" s="59"/>
+      <c r="P33" s="60"/>
     </row>
     <row r="34" spans="2:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="123"/>
-      <c r="C34" s="124"/>
-      <c r="D34" s="124"/>
-      <c r="E34" s="124"/>
-      <c r="F34" s="124"/>
-      <c r="G34" s="124"/>
-      <c r="H34" s="124"/>
-      <c r="I34" s="124"/>
-      <c r="J34" s="125"/>
-      <c r="K34" s="43"/>
-      <c r="L34" s="126" t="s">
+      <c r="B34" s="61"/>
+      <c r="C34" s="62"/>
+      <c r="D34" s="62"/>
+      <c r="E34" s="62"/>
+      <c r="F34" s="62"/>
+      <c r="G34" s="62"/>
+      <c r="H34" s="62"/>
+      <c r="I34" s="62"/>
+      <c r="J34" s="63"/>
+      <c r="K34" s="36"/>
+      <c r="L34" s="64" t="s">
         <v>25</v>
       </c>
-      <c r="M34" s="44" t="s">
-        <v>61</v>
-      </c>
-      <c r="N34" s="44"/>
+      <c r="M34" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="N34" s="37"/>
       <c r="P34" s="9"/>
     </row>
     <row r="35" spans="2:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="123"/>
-      <c r="C35" s="124"/>
-      <c r="D35" s="124"/>
-      <c r="E35" s="124"/>
-      <c r="F35" s="124"/>
-      <c r="G35" s="124"/>
-      <c r="H35" s="124"/>
-      <c r="I35" s="124"/>
-      <c r="J35" s="125"/>
-      <c r="K35" s="45"/>
-      <c r="L35" s="127"/>
-      <c r="M35" s="46" t="s">
-        <v>62</v>
-      </c>
-      <c r="N35" s="46"/>
+      <c r="B35" s="61"/>
+      <c r="C35" s="62"/>
+      <c r="D35" s="62"/>
+      <c r="E35" s="62"/>
+      <c r="F35" s="62"/>
+      <c r="G35" s="62"/>
+      <c r="H35" s="62"/>
+      <c r="I35" s="62"/>
+      <c r="J35" s="63"/>
+      <c r="K35" s="38"/>
+      <c r="L35" s="65"/>
+      <c r="M35" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="N35" s="39"/>
       <c r="O35" s="7"/>
-      <c r="P35" s="47"/>
+      <c r="P35" s="40"/>
     </row>
     <row r="36" spans="2:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="2"/>
       <c r="P36" s="9"/>
     </row>
     <row r="37" spans="2:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="129" t="s">
+      <c r="B37" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="C37" s="130"/>
-      <c r="D37" s="130"/>
-      <c r="E37" s="130"/>
-      <c r="F37" s="130"/>
-      <c r="G37" s="131"/>
+      <c r="C37" s="52"/>
+      <c r="D37" s="52"/>
+      <c r="E37" s="52"/>
+      <c r="F37" s="52"/>
+      <c r="G37" s="53"/>
       <c r="H37" s="4"/>
-      <c r="J37" s="30"/>
-      <c r="K37" s="30"/>
-      <c r="L37" s="119" t="s">
-        <v>54</v>
-      </c>
-      <c r="M37" s="119"/>
-      <c r="N37" s="119"/>
-      <c r="O37" s="119"/>
-      <c r="P37" s="119"/>
+      <c r="J37" s="23"/>
+      <c r="K37" s="23"/>
+      <c r="L37" s="54" t="s">
+        <v>53</v>
+      </c>
+      <c r="M37" s="54"/>
+      <c r="N37" s="54"/>
+      <c r="O37" s="54"/>
+      <c r="P37" s="54"/>
     </row>
     <row r="38" spans="2:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="129" t="s">
+      <c r="B38" s="51" t="s">
         <v>52</v>
       </c>
-      <c r="C38" s="130"/>
-      <c r="D38" s="130"/>
-      <c r="E38" s="130"/>
-      <c r="F38" s="130"/>
-      <c r="G38" s="131"/>
+      <c r="C38" s="52"/>
+      <c r="D38" s="52"/>
+      <c r="E38" s="52"/>
+      <c r="F38" s="52"/>
+      <c r="G38" s="53"/>
       <c r="H38" s="4"/>
-      <c r="J38" s="30"/>
-      <c r="K38" s="30"/>
-      <c r="L38" s="119" t="s">
-        <v>55</v>
-      </c>
-      <c r="M38" s="119"/>
-      <c r="N38" s="119"/>
-      <c r="O38" s="119"/>
-      <c r="P38" s="119"/>
+      <c r="J38" s="23"/>
+      <c r="K38" s="23"/>
+      <c r="L38" s="54" t="s">
+        <v>54</v>
+      </c>
+      <c r="M38" s="54"/>
+      <c r="N38" s="54"/>
+      <c r="O38" s="54"/>
+      <c r="P38" s="54"/>
     </row>
     <row r="39" spans="2:16" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="132" t="s">
-        <v>53</v>
-      </c>
-      <c r="C39" s="133"/>
-      <c r="D39" s="133"/>
-      <c r="E39" s="133"/>
-      <c r="F39" s="133"/>
-      <c r="G39" s="134"/>
-      <c r="H39" s="48"/>
-      <c r="I39" s="49"/>
-      <c r="J39" s="50"/>
-      <c r="K39" s="51"/>
-      <c r="L39" s="120" t="s">
-        <v>56</v>
-      </c>
-      <c r="M39" s="120"/>
-      <c r="N39" s="120"/>
-      <c r="O39" s="120"/>
-      <c r="P39" s="120"/>
+      <c r="B39" s="55" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="56"/>
+      <c r="D39" s="56"/>
+      <c r="E39" s="56"/>
+      <c r="F39" s="56"/>
+      <c r="G39" s="57"/>
+      <c r="H39" s="41"/>
+      <c r="I39" s="42"/>
+      <c r="J39" s="43"/>
+      <c r="K39" s="44"/>
+      <c r="L39" s="58" t="s">
+        <v>66</v>
+      </c>
+      <c r="M39" s="58"/>
+      <c r="N39" s="58"/>
+      <c r="O39" s="58"/>
+      <c r="P39" s="58"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="46">
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="L38:P38"/>
-    <mergeCell ref="B39:G39"/>
-    <mergeCell ref="L39:P39"/>
-    <mergeCell ref="L33:P33"/>
-    <mergeCell ref="B34:J34"/>
-    <mergeCell ref="L34:L35"/>
-    <mergeCell ref="B35:J35"/>
-    <mergeCell ref="B37:G37"/>
-    <mergeCell ref="L37:P37"/>
-    <mergeCell ref="B33:J33"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="B3:C6"/>
+    <mergeCell ref="D3:M6"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="C13:E16"/>
+    <mergeCell ref="F13:F16"/>
+    <mergeCell ref="G13:G16"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="E9:I10"/>
+    <mergeCell ref="J10:M10"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="K13:M13"/>
     <mergeCell ref="N13:P13"/>
@@ -3809,22 +3814,22 @@
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C20:E20"/>
     <mergeCell ref="C21:E21"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="E9:I10"/>
-    <mergeCell ref="J10:M10"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="C13:E16"/>
-    <mergeCell ref="F13:F16"/>
-    <mergeCell ref="G13:G16"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="B3:C6"/>
-    <mergeCell ref="D3:M6"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="L38:P38"/>
+    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="L39:P39"/>
+    <mergeCell ref="L33:P33"/>
+    <mergeCell ref="B34:J34"/>
+    <mergeCell ref="L34:L35"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="L37:P37"/>
+    <mergeCell ref="B33:J33"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.70866141732283472" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>

<commit_message>
Importaciones de Almacen ADV realizado de forma manual en dbeaver y procesado en filament
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO SUM COTIZACIONES.xlsx
+++ b/storage/app/templates/FORMATO SUM COTIZACIONES.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA-OFICIAL-AGARCORP\storage\app\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adv\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{559E1C37-2D23-4DAE-80C6-B8CC2A8C2AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E483495B-67D6-41D9-93E6-FB6F316CAD52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{309D63E5-5CD5-46E5-9FEC-D63E43A25BAB}"/>
   </bookViews>
@@ -1114,9 +1114,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1159,53 +1156,159 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="22"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="22"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="22"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="22"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="22"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="22"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="22"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="22"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="22"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="16"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="8"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="8"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1219,6 +1322,45 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1231,198 +1373,56 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="16"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="8"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="8"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="22"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="22"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="22"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="22"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="22"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="22"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="22"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="22"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="22"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2842,82 +2842,82 @@
   <sheetData>
     <row r="2" spans="2:16" ht="15.6" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="122"/>
-      <c r="C3" s="123"/>
-      <c r="D3" s="128" t="s">
+      <c r="B3" s="59"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="E3" s="129"/>
-      <c r="F3" s="129"/>
-      <c r="G3" s="129"/>
-      <c r="H3" s="129"/>
-      <c r="I3" s="129"/>
-      <c r="J3" s="129"/>
-      <c r="K3" s="129"/>
-      <c r="L3" s="129"/>
-      <c r="M3" s="130"/>
-      <c r="N3" s="137" t="s">
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="66"/>
+      <c r="K3" s="66"/>
+      <c r="L3" s="66"/>
+      <c r="M3" s="67"/>
+      <c r="N3" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="O3" s="138"/>
-      <c r="P3" s="139"/>
+      <c r="O3" s="75"/>
+      <c r="P3" s="76"/>
     </row>
     <row r="4" spans="2:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="124"/>
-      <c r="C4" s="125"/>
-      <c r="D4" s="131"/>
-      <c r="E4" s="132"/>
-      <c r="F4" s="132"/>
-      <c r="G4" s="132"/>
-      <c r="H4" s="132"/>
-      <c r="I4" s="132"/>
-      <c r="J4" s="132"/>
-      <c r="K4" s="132"/>
-      <c r="L4" s="132"/>
-      <c r="M4" s="133"/>
-      <c r="N4" s="140" t="s">
+      <c r="B4" s="61"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="69"/>
+      <c r="J4" s="69"/>
+      <c r="K4" s="69"/>
+      <c r="L4" s="69"/>
+      <c r="M4" s="70"/>
+      <c r="N4" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="O4" s="141"/>
-      <c r="P4" s="142"/>
+      <c r="O4" s="78"/>
+      <c r="P4" s="79"/>
     </row>
     <row r="5" spans="2:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="124"/>
-      <c r="C5" s="125"/>
-      <c r="D5" s="131"/>
-      <c r="E5" s="132"/>
-      <c r="F5" s="132"/>
-      <c r="G5" s="132"/>
-      <c r="H5" s="132"/>
-      <c r="I5" s="132"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="132"/>
-      <c r="L5" s="132"/>
-      <c r="M5" s="133"/>
-      <c r="N5" s="140" t="s">
+      <c r="B5" s="61"/>
+      <c r="C5" s="62"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="69"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="69"/>
+      <c r="I5" s="69"/>
+      <c r="J5" s="69"/>
+      <c r="K5" s="69"/>
+      <c r="L5" s="69"/>
+      <c r="M5" s="70"/>
+      <c r="N5" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="O5" s="141"/>
-      <c r="P5" s="142"/>
+      <c r="O5" s="78"/>
+      <c r="P5" s="79"/>
     </row>
     <row r="6" spans="2:16" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="126"/>
-      <c r="C6" s="127"/>
-      <c r="D6" s="134"/>
-      <c r="E6" s="135"/>
-      <c r="F6" s="135"/>
-      <c r="G6" s="135"/>
-      <c r="H6" s="135"/>
-      <c r="I6" s="135"/>
-      <c r="J6" s="135"/>
-      <c r="K6" s="135"/>
-      <c r="L6" s="135"/>
-      <c r="M6" s="136"/>
-      <c r="N6" s="143" t="s">
+      <c r="B6" s="63"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="71"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="72"/>
+      <c r="H6" s="72"/>
+      <c r="I6" s="72"/>
+      <c r="J6" s="72"/>
+      <c r="K6" s="72"/>
+      <c r="L6" s="72"/>
+      <c r="M6" s="73"/>
+      <c r="N6" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="O6" s="144"/>
-      <c r="P6" s="145"/>
+      <c r="O6" s="81"/>
+      <c r="P6" s="82"/>
     </row>
     <row r="7" spans="2:16" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
@@ -2936,56 +2936,56 @@
       <c r="P7" s="5"/>
     </row>
     <row r="8" spans="2:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="95" t="s">
+      <c r="B8" s="102" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="96"/>
-      <c r="D8" s="97" t="s">
+      <c r="C8" s="103"/>
+      <c r="D8" s="104" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="97"/>
-      <c r="F8" s="97"/>
-      <c r="G8" s="97"/>
+      <c r="E8" s="104"/>
+      <c r="F8" s="104"/>
+      <c r="G8" s="104"/>
       <c r="H8" s="6"/>
       <c r="I8" s="7"/>
       <c r="M8" s="8" t="s">
         <v>6</v>
       </c>
       <c r="N8" s="8"/>
-      <c r="O8" s="98" t="s">
+      <c r="O8" s="105" t="s">
         <v>27</v>
       </c>
-      <c r="P8" s="99"/>
+      <c r="P8" s="106"/>
     </row>
     <row r="9" spans="2:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="54"/>
-      <c r="C9" s="59"/>
-      <c r="E9" s="100" t="s">
+      <c r="B9" s="53"/>
+      <c r="C9" s="58"/>
+      <c r="E9" s="107" t="s">
         <v>28</v>
       </c>
-      <c r="F9" s="100"/>
-      <c r="G9" s="100"/>
-      <c r="H9" s="100"/>
-      <c r="I9" s="100"/>
+      <c r="F9" s="107"/>
+      <c r="G9" s="107"/>
+      <c r="H9" s="107"/>
+      <c r="I9" s="107"/>
       <c r="P9" s="9"/>
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B10" s="54" t="s">
+      <c r="B10" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="59"/>
+      <c r="C10" s="58"/>
       <c r="D10" s="10"/>
-      <c r="E10" s="101"/>
-      <c r="F10" s="101"/>
-      <c r="G10" s="101"/>
-      <c r="H10" s="101"/>
-      <c r="I10" s="101"/>
-      <c r="J10" s="102" t="s">
+      <c r="E10" s="108"/>
+      <c r="F10" s="108"/>
+      <c r="G10" s="108"/>
+      <c r="H10" s="108"/>
+      <c r="I10" s="108"/>
+      <c r="J10" s="109" t="s">
         <v>8</v>
       </c>
-      <c r="K10" s="102"/>
-      <c r="L10" s="102"/>
-      <c r="M10" s="102"/>
+      <c r="K10" s="109"/>
+      <c r="L10" s="109"/>
+      <c r="M10" s="109"/>
       <c r="N10" s="8"/>
       <c r="O10" s="1" t="s">
         <v>56</v>
@@ -3004,67 +3004,67 @@
       <c r="P12" s="9"/>
     </row>
     <row r="13" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="103" t="s">
+      <c r="B13" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="104" t="s">
+      <c r="C13" s="84" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="105"/>
-      <c r="E13" s="106"/>
-      <c r="F13" s="113" t="s">
+      <c r="D13" s="85"/>
+      <c r="E13" s="86"/>
+      <c r="F13" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="116" t="s">
+      <c r="G13" s="96" t="s">
         <v>12</v>
       </c>
-      <c r="H13" s="119" t="s">
+      <c r="H13" s="99" t="s">
         <v>13</v>
       </c>
-      <c r="I13" s="120"/>
-      <c r="J13" s="121"/>
-      <c r="K13" s="82" t="s">
+      <c r="I13" s="100"/>
+      <c r="J13" s="101"/>
+      <c r="K13" s="113" t="s">
         <v>13</v>
       </c>
-      <c r="L13" s="83"/>
-      <c r="M13" s="84"/>
-      <c r="N13" s="85" t="s">
+      <c r="L13" s="114"/>
+      <c r="M13" s="115"/>
+      <c r="N13" s="116" t="s">
         <v>13</v>
       </c>
-      <c r="O13" s="86"/>
-      <c r="P13" s="87"/>
+      <c r="O13" s="117"/>
+      <c r="P13" s="118"/>
     </row>
     <row r="14" spans="2:16" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="103"/>
-      <c r="C14" s="107"/>
-      <c r="D14" s="108"/>
-      <c r="E14" s="109"/>
-      <c r="F14" s="114"/>
-      <c r="G14" s="117"/>
-      <c r="H14" s="88" t="s">
+      <c r="B14" s="83"/>
+      <c r="C14" s="87"/>
+      <c r="D14" s="88"/>
+      <c r="E14" s="89"/>
+      <c r="F14" s="94"/>
+      <c r="G14" s="97"/>
+      <c r="H14" s="119" t="s">
         <v>29</v>
       </c>
-      <c r="I14" s="89"/>
-      <c r="J14" s="90"/>
-      <c r="K14" s="88" t="s">
+      <c r="I14" s="120"/>
+      <c r="J14" s="121"/>
+      <c r="K14" s="119" t="s">
         <v>31</v>
       </c>
-      <c r="L14" s="89"/>
-      <c r="M14" s="90"/>
-      <c r="N14" s="88" t="s">
+      <c r="L14" s="120"/>
+      <c r="M14" s="121"/>
+      <c r="N14" s="119" t="s">
         <v>30</v>
       </c>
-      <c r="O14" s="89"/>
-      <c r="P14" s="90"/>
+      <c r="O14" s="120"/>
+      <c r="P14" s="121"/>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B15" s="103"/>
-      <c r="C15" s="107"/>
-      <c r="D15" s="108"/>
-      <c r="E15" s="109"/>
-      <c r="F15" s="114"/>
-      <c r="G15" s="117"/>
-      <c r="H15" s="91" t="s">
+      <c r="B15" s="83"/>
+      <c r="C15" s="87"/>
+      <c r="D15" s="88"/>
+      <c r="E15" s="89"/>
+      <c r="F15" s="94"/>
+      <c r="G15" s="97"/>
+      <c r="H15" s="122" t="s">
         <v>14</v>
       </c>
       <c r="I15" s="12" t="s">
@@ -3073,51 +3073,51 @@
       <c r="J15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="K15" s="93" t="s">
+      <c r="K15" s="124" t="s">
         <v>14</v>
       </c>
-      <c r="L15" s="46" t="s">
+      <c r="L15" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="M15" s="47" t="s">
+      <c r="M15" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="N15" s="93" t="s">
+      <c r="N15" s="124" t="s">
         <v>14</v>
       </c>
       <c r="O15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="P15" s="48" t="s">
+      <c r="P15" s="47" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B16" s="103"/>
-      <c r="C16" s="110"/>
-      <c r="D16" s="111"/>
-      <c r="E16" s="112"/>
-      <c r="F16" s="115"/>
-      <c r="G16" s="118"/>
-      <c r="H16" s="92"/>
+      <c r="B16" s="83"/>
+      <c r="C16" s="90"/>
+      <c r="D16" s="91"/>
+      <c r="E16" s="92"/>
+      <c r="F16" s="95"/>
+      <c r="G16" s="98"/>
+      <c r="H16" s="123"/>
       <c r="I16" s="13" t="s">
         <v>17</v>
       </c>
       <c r="J16" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="K16" s="94"/>
+      <c r="K16" s="125"/>
       <c r="L16" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="M16" s="49" t="s">
+      <c r="M16" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="N16" s="94"/>
+      <c r="N16" s="125"/>
       <c r="O16" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="P16" s="50" t="s">
+      <c r="P16" s="49" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3125,11 +3125,11 @@
       <c r="B17" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="76" t="s">
+      <c r="C17" s="110" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="77"/>
-      <c r="E17" s="78"/>
+      <c r="D17" s="111"/>
+      <c r="E17" s="112"/>
       <c r="F17" s="15" t="s">
         <v>63</v>
       </c>
@@ -3157,7 +3157,7 @@
       <c r="N17" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O17" s="45" t="s">
+      <c r="O17" s="145" t="s">
         <v>40</v>
       </c>
       <c r="P17" s="18" t="s">
@@ -3168,11 +3168,11 @@
       <c r="B18" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C18" s="76" t="s">
+      <c r="C18" s="110" t="s">
         <v>62</v>
       </c>
-      <c r="D18" s="77"/>
-      <c r="E18" s="78"/>
+      <c r="D18" s="111"/>
+      <c r="E18" s="112"/>
       <c r="F18" s="15" t="s">
         <v>63</v>
       </c>
@@ -3200,7 +3200,7 @@
       <c r="N18" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O18" s="45" t="s">
+      <c r="O18" s="145" t="s">
         <v>40</v>
       </c>
       <c r="P18" s="18" t="s">
@@ -3214,11 +3214,11 @@
       <c r="B19" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="76" t="s">
+      <c r="C19" s="110" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="77"/>
-      <c r="E19" s="78"/>
+      <c r="D19" s="111"/>
+      <c r="E19" s="112"/>
       <c r="F19" s="15" t="s">
         <v>63</v>
       </c>
@@ -3246,7 +3246,7 @@
       <c r="N19" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O19" s="45" t="s">
+      <c r="O19" s="145" t="s">
         <v>40</v>
       </c>
       <c r="P19" s="18" t="s">
@@ -3257,11 +3257,11 @@
       <c r="B20" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="76" t="s">
+      <c r="C20" s="110" t="s">
         <v>62</v>
       </c>
-      <c r="D20" s="77"/>
-      <c r="E20" s="78"/>
+      <c r="D20" s="111"/>
+      <c r="E20" s="112"/>
       <c r="F20" s="15" t="s">
         <v>63</v>
       </c>
@@ -3289,7 +3289,7 @@
       <c r="N20" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O20" s="45" t="s">
+      <c r="O20" s="145" t="s">
         <v>40</v>
       </c>
       <c r="P20" s="18" t="s">
@@ -3300,11 +3300,11 @@
       <c r="B21" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C21" s="76" t="s">
+      <c r="C21" s="110" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="77"/>
-      <c r="E21" s="78"/>
+      <c r="D21" s="111"/>
+      <c r="E21" s="112"/>
       <c r="F21" s="15" t="s">
         <v>63</v>
       </c>
@@ -3332,7 +3332,7 @@
       <c r="N21" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O21" s="45" t="s">
+      <c r="O21" s="145" t="s">
         <v>40</v>
       </c>
       <c r="P21" s="18" t="s">
@@ -3343,11 +3343,11 @@
       <c r="B22" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C22" s="76" t="s">
+      <c r="C22" s="110" t="s">
         <v>62</v>
       </c>
-      <c r="D22" s="77"/>
-      <c r="E22" s="78"/>
+      <c r="D22" s="111"/>
+      <c r="E22" s="112"/>
       <c r="F22" s="15" t="s">
         <v>63</v>
       </c>
@@ -3375,7 +3375,7 @@
       <c r="N22" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O22" s="45" t="s">
+      <c r="O22" s="145" t="s">
         <v>40</v>
       </c>
       <c r="P22" s="18" t="s">
@@ -3386,11 +3386,11 @@
       <c r="B23" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C23" s="76" t="s">
+      <c r="C23" s="110" t="s">
         <v>62</v>
       </c>
-      <c r="D23" s="77"/>
-      <c r="E23" s="78"/>
+      <c r="D23" s="111"/>
+      <c r="E23" s="112"/>
       <c r="F23" s="15" t="s">
         <v>63</v>
       </c>
@@ -3418,7 +3418,7 @@
       <c r="N23" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O23" s="45" t="s">
+      <c r="O23" s="145" t="s">
         <v>40</v>
       </c>
       <c r="P23" s="18" t="s">
@@ -3429,11 +3429,11 @@
       <c r="B24" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C24" s="76" t="s">
+      <c r="C24" s="110" t="s">
         <v>62</v>
       </c>
-      <c r="D24" s="77"/>
-      <c r="E24" s="78"/>
+      <c r="D24" s="111"/>
+      <c r="E24" s="112"/>
       <c r="F24" s="15" t="s">
         <v>63</v>
       </c>
@@ -3461,7 +3461,7 @@
       <c r="N24" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O24" s="45" t="s">
+      <c r="O24" s="145" t="s">
         <v>40</v>
       </c>
       <c r="P24" s="18" t="s">
@@ -3473,11 +3473,11 @@
       <c r="B25" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="76" t="s">
+      <c r="C25" s="110" t="s">
         <v>62</v>
       </c>
-      <c r="D25" s="77"/>
-      <c r="E25" s="78"/>
+      <c r="D25" s="111"/>
+      <c r="E25" s="112"/>
       <c r="F25" s="15" t="s">
         <v>63</v>
       </c>
@@ -3505,7 +3505,7 @@
       <c r="N25" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O25" s="45" t="s">
+      <c r="O25" s="145" t="s">
         <v>40</v>
       </c>
       <c r="P25" s="18" t="s">
@@ -3516,11 +3516,11 @@
       <c r="B26" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C26" s="76" t="s">
+      <c r="C26" s="110" t="s">
         <v>62</v>
       </c>
-      <c r="D26" s="77"/>
-      <c r="E26" s="78"/>
+      <c r="D26" s="111"/>
+      <c r="E26" s="112"/>
       <c r="F26" s="15" t="s">
         <v>63</v>
       </c>
@@ -3548,7 +3548,7 @@
       <c r="N26" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O26" s="45" t="s">
+      <c r="O26" s="145" t="s">
         <v>40</v>
       </c>
       <c r="P26" s="18" t="s">
@@ -3559,11 +3559,11 @@
       <c r="B27" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="79" t="s">
+      <c r="C27" s="126" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="80"/>
-      <c r="E27" s="81"/>
+      <c r="D27" s="127"/>
+      <c r="E27" s="128"/>
       <c r="F27" s="15" t="s">
         <v>63</v>
       </c>
@@ -3591,7 +3591,7 @@
       <c r="N27" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="O27" s="45" t="s">
+      <c r="O27" s="145" t="s">
         <v>40</v>
       </c>
       <c r="P27" s="18" t="s">
@@ -3604,7 +3604,7 @@
       <c r="P28" s="9"/>
     </row>
     <row r="29" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="54" t="s">
+      <c r="B29" s="53" t="s">
         <v>20</v>
       </c>
       <c r="G29" s="23"/>
@@ -3677,59 +3677,59 @@
       <c r="P32" s="9"/>
     </row>
     <row r="33" spans="2:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="75" t="s">
+      <c r="B33" s="144" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="71"/>
-      <c r="D33" s="71"/>
-      <c r="E33" s="71"/>
-      <c r="F33" s="71"/>
-      <c r="G33" s="71"/>
-      <c r="H33" s="71"/>
-      <c r="I33" s="71"/>
-      <c r="J33" s="72"/>
+      <c r="C33" s="140"/>
+      <c r="D33" s="140"/>
+      <c r="E33" s="140"/>
+      <c r="F33" s="140"/>
+      <c r="G33" s="140"/>
+      <c r="H33" s="140"/>
+      <c r="I33" s="140"/>
+      <c r="J33" s="141"/>
       <c r="K33" s="35"/>
-      <c r="L33" s="68" t="s">
+      <c r="L33" s="137" t="s">
         <v>24</v>
       </c>
-      <c r="M33" s="68"/>
-      <c r="N33" s="68"/>
-      <c r="O33" s="68"/>
-      <c r="P33" s="69"/>
+      <c r="M33" s="137"/>
+      <c r="N33" s="137"/>
+      <c r="O33" s="137"/>
+      <c r="P33" s="138"/>
     </row>
     <row r="34" spans="2:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="70"/>
-      <c r="C34" s="71"/>
-      <c r="D34" s="71"/>
-      <c r="E34" s="71"/>
-      <c r="F34" s="71"/>
-      <c r="G34" s="71"/>
-      <c r="H34" s="71"/>
-      <c r="I34" s="71"/>
-      <c r="J34" s="72"/>
+      <c r="B34" s="139"/>
+      <c r="C34" s="140"/>
+      <c r="D34" s="140"/>
+      <c r="E34" s="140"/>
+      <c r="F34" s="140"/>
+      <c r="G34" s="140"/>
+      <c r="H34" s="140"/>
+      <c r="I34" s="140"/>
+      <c r="J34" s="141"/>
       <c r="K34" s="36"/>
-      <c r="L34" s="73" t="s">
+      <c r="L34" s="142" t="s">
         <v>25</v>
       </c>
-      <c r="M34" s="52" t="s">
+      <c r="M34" s="51" t="s">
         <v>59</v>
       </c>
       <c r="N34" s="37"/>
       <c r="P34" s="9"/>
     </row>
     <row r="35" spans="2:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="70"/>
-      <c r="C35" s="71"/>
-      <c r="D35" s="71"/>
-      <c r="E35" s="71"/>
-      <c r="F35" s="71"/>
-      <c r="G35" s="71"/>
-      <c r="H35" s="71"/>
-      <c r="I35" s="71"/>
-      <c r="J35" s="72"/>
+      <c r="B35" s="139"/>
+      <c r="C35" s="140"/>
+      <c r="D35" s="140"/>
+      <c r="E35" s="140"/>
+      <c r="F35" s="140"/>
+      <c r="G35" s="140"/>
+      <c r="H35" s="140"/>
+      <c r="I35" s="140"/>
+      <c r="J35" s="141"/>
       <c r="K35" s="38"/>
-      <c r="L35" s="74"/>
-      <c r="M35" s="53" t="s">
+      <c r="L35" s="143"/>
+      <c r="M35" s="52" t="s">
         <v>60</v>
       </c>
       <c r="N35" s="39"/>
@@ -3741,105 +3741,105 @@
       <c r="P36" s="9"/>
     </row>
     <row r="37" spans="2:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="60" t="s">
+      <c r="B37" s="129" t="s">
         <v>51</v>
       </c>
-      <c r="C37" s="61"/>
-      <c r="D37" s="61"/>
-      <c r="E37" s="61"/>
-      <c r="F37" s="61"/>
-      <c r="G37" s="62"/>
+      <c r="C37" s="130"/>
+      <c r="D37" s="130"/>
+      <c r="E37" s="130"/>
+      <c r="F37" s="130"/>
+      <c r="G37" s="131"/>
       <c r="H37" s="4"/>
       <c r="J37" s="23"/>
       <c r="K37" s="23"/>
-      <c r="L37" s="63" t="s">
+      <c r="L37" s="132" t="s">
         <v>53</v>
       </c>
-      <c r="M37" s="63"/>
-      <c r="N37" s="63"/>
-      <c r="O37" s="63"/>
-      <c r="P37" s="63"/>
+      <c r="M37" s="132"/>
+      <c r="N37" s="132"/>
+      <c r="O37" s="132"/>
+      <c r="P37" s="132"/>
     </row>
     <row r="38" spans="2:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="60" t="s">
+      <c r="B38" s="129" t="s">
         <v>52</v>
       </c>
-      <c r="C38" s="61"/>
-      <c r="D38" s="61"/>
-      <c r="E38" s="61"/>
-      <c r="F38" s="61"/>
-      <c r="G38" s="62"/>
+      <c r="C38" s="130"/>
+      <c r="D38" s="130"/>
+      <c r="E38" s="130"/>
+      <c r="F38" s="130"/>
+      <c r="G38" s="131"/>
       <c r="H38" s="4"/>
       <c r="J38" s="23"/>
       <c r="K38" s="23"/>
-      <c r="L38" s="63" t="s">
+      <c r="L38" s="132" t="s">
         <v>54</v>
       </c>
-      <c r="M38" s="63"/>
-      <c r="N38" s="63"/>
-      <c r="O38" s="63"/>
-      <c r="P38" s="63"/>
+      <c r="M38" s="132"/>
+      <c r="N38" s="132"/>
+      <c r="O38" s="132"/>
+      <c r="P38" s="132"/>
     </row>
     <row r="39" spans="2:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="58"/>
-      <c r="C39" s="56"/>
-      <c r="D39" s="56" t="s">
+      <c r="B39" s="57"/>
+      <c r="C39" s="55"/>
+      <c r="D39" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="E39" s="56"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="57"/>
-      <c r="H39" s="51"/>
+      <c r="E39" s="55"/>
+      <c r="F39" s="55"/>
+      <c r="G39" s="56"/>
+      <c r="H39" s="50"/>
       <c r="J39" s="23"/>
       <c r="K39" s="23"/>
-      <c r="L39" s="55"/>
-      <c r="M39" s="56" t="s">
+      <c r="L39" s="54"/>
+      <c r="M39" s="55" t="s">
         <v>66</v>
       </c>
-      <c r="N39" s="56"/>
-      <c r="O39" s="56"/>
-      <c r="P39" s="57"/>
+      <c r="N39" s="55"/>
+      <c r="O39" s="55"/>
+      <c r="P39" s="56"/>
     </row>
     <row r="40" spans="2:16" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="64" t="s">
+      <c r="B40" s="133" t="s">
         <v>65</v>
       </c>
-      <c r="C40" s="65"/>
-      <c r="D40" s="65"/>
-      <c r="E40" s="65"/>
-      <c r="F40" s="65"/>
-      <c r="G40" s="66"/>
+      <c r="C40" s="134"/>
+      <c r="D40" s="134"/>
+      <c r="E40" s="134"/>
+      <c r="F40" s="134"/>
+      <c r="G40" s="135"/>
       <c r="H40" s="41"/>
       <c r="I40" s="42"/>
       <c r="J40" s="43"/>
       <c r="K40" s="44"/>
-      <c r="L40" s="67" t="s">
+      <c r="L40" s="136" t="s">
         <v>67</v>
       </c>
-      <c r="M40" s="67"/>
-      <c r="N40" s="67"/>
-      <c r="O40" s="67"/>
-      <c r="P40" s="67"/>
+      <c r="M40" s="136"/>
+      <c r="N40" s="136"/>
+      <c r="O40" s="136"/>
+      <c r="P40" s="136"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="46">
-    <mergeCell ref="B3:C6"/>
-    <mergeCell ref="D3:M6"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="C13:E16"/>
-    <mergeCell ref="F13:F16"/>
-    <mergeCell ref="G13:G16"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="E9:I10"/>
-    <mergeCell ref="J10:M10"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="L38:P38"/>
+    <mergeCell ref="B40:G40"/>
+    <mergeCell ref="L40:P40"/>
+    <mergeCell ref="L33:P33"/>
+    <mergeCell ref="B34:J34"/>
+    <mergeCell ref="L34:L35"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="L37:P37"/>
+    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C27:E27"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="K13:M13"/>
     <mergeCell ref="N13:P13"/>
@@ -3854,22 +3854,22 @@
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C20:E20"/>
     <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="L38:P38"/>
-    <mergeCell ref="B40:G40"/>
-    <mergeCell ref="L40:P40"/>
-    <mergeCell ref="L33:P33"/>
-    <mergeCell ref="B34:J34"/>
-    <mergeCell ref="L34:L35"/>
-    <mergeCell ref="B35:J35"/>
-    <mergeCell ref="B37:G37"/>
-    <mergeCell ref="L37:P37"/>
-    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="E9:I10"/>
+    <mergeCell ref="J10:M10"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="C13:E16"/>
+    <mergeCell ref="F13:F16"/>
+    <mergeCell ref="G13:G16"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="B3:C6"/>
+    <mergeCell ref="D3:M6"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="N6:P6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.70866141732283472" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>